<commit_message>
feat: Criação do perfil de Mentor com Stored Procedure
</commit_message>
<xml_diff>
--- a/api/desempenho/2025-07-04.xlsx
+++ b/api/desempenho/2025-07-04.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -728,6 +728,146 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2025-07-04</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>14:31:03</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>39673</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>80.83</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota Mentorship Profiles</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2025-07-04</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>14:31:29</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>39750</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>80.98999999999999</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota Mentorship Profiles</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2025-07-04</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>14:32:10</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>39826</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>81.02</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota Mentorship Profiles</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2025-07-04</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>14:32:50</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>39894</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>81.05</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota Users</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2025-07-04</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>14:33:16</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>39953</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>81.14</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota Mentorship Profiles</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: Refatoração do código
</commit_message>
<xml_diff>
--- a/api/desempenho/2025-07-04.xlsx
+++ b/api/desempenho/2025-07-04.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,6 +471,62 @@
         <v>80.31999999999999</v>
       </c>
       <c r="F2" t="inlineStr">
+        <is>
+          <t>Acessou a rota Mentorship Profiles</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2025-07-04</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>18:30:14</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>23809</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>80.48999999999999</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Acesso na rota UserTechStacks</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2025-07-04</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>18:33:42</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>24340</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>80.68000000000001</v>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>Acessou a rota Mentorship Profiles</t>
         </is>

</xml_diff>